<commit_message>
feat: Update product data in sample dataset
</commit_message>
<xml_diff>
--- a/sample_data/products.xlsx
+++ b/sample_data/products.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -483,6 +483,11 @@
           <t>hsn_code</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>other_barcodes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -517,7 +522,11 @@
       <c r="H2" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>8901000000101, 8901000000102</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -552,7 +561,6 @@
       <c r="H3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -587,7 +595,6 @@
       <c r="H4" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -622,7 +629,6 @@
       <c r="H5" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -657,7 +663,6 @@
       <c r="H6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -692,7 +697,6 @@
       <c r="H7" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -727,7 +731,6 @@
       <c r="H8" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -762,7 +765,6 @@
       <c r="H9" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -797,7 +799,6 @@
       <c r="H10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -832,7 +833,6 @@
       <c r="H11" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -867,7 +867,6 @@
       <c r="H12" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -902,7 +901,6 @@
       <c r="H13" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -937,7 +935,6 @@
       <c r="H14" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -972,7 +969,6 @@
       <c r="H15" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1007,7 +1003,6 @@
       <c r="H16" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1042,7 +1037,6 @@
       <c r="H17" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1077,7 +1071,6 @@
       <c r="H18" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1112,7 +1105,6 @@
       <c r="H19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1147,7 +1139,6 @@
       <c r="H20" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1182,7 +1173,6 @@
       <c r="H21" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>